<commit_message>
Perfil Servidor: minha área, envio pedido pelo gerente e validação de bens
- Novo perfil "servidor" (Paula Menezes = quem envia, Diego Santos = quem
  recebe). A API só libera para ele as rotas marcadas com `servidor: true`
  (próprio perfil, minha área, envio/recebimento das movimentações em que
  participa); todo o resto responde 403.
- GET /me/area: bens no nome da pessoa + tarefas (enviar, receber, validar).
- Validação de bens (VAL-AAAA-NNNN): o gerente pede, a pessoa responde
  "está comigo"/"não está"; "não está" vira pendência de não localizado.
- Gerente que pede uma movimentação e se indica como aprovador já a aprova
  (ele gerou a necessidade).
- "Entrega" passa a se chamar "Envio" em todo texto visível (telas, PDF,
  mensagens, histórico). Nomes internos e campos da API não mudam.
- Planilha de exemplo com bens no nome dos servidores.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/novos_itens_predio_sede.xlsx
+++ b/sample-data/novos_itens_predio_sede.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>Nº Tombamento</t>
   </si>
@@ -67,85 +67,91 @@
     <t>Secretaria de Informática</t>
   </si>
   <si>
+    <t>Paula Menezes</t>
+  </si>
+  <si>
+    <t>Novo</t>
+  </si>
+  <si>
+    <t>15/10/2026</t>
+  </si>
+  <si>
+    <t>6.290,00</t>
+  </si>
+  <si>
+    <t>0200002</t>
+  </si>
+  <si>
+    <t>DLT5440A02</t>
+  </si>
+  <si>
+    <t>Diego Santos</t>
+  </si>
+  <si>
+    <t>0200003</t>
+  </si>
+  <si>
+    <t>Cadeira giratória ergonômica com braços</t>
+  </si>
+  <si>
+    <t>Mobiliário</t>
+  </si>
+  <si>
+    <t>Cavaletti</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Secretaria de Administração</t>
+  </si>
+  <si>
+    <t>Bom</t>
+  </si>
+  <si>
+    <t>03/03/2025</t>
+  </si>
+  <si>
+    <t>890,00</t>
+  </si>
+  <si>
+    <t>0200004</t>
+  </si>
+  <si>
+    <t>Projetor multimídia Epson PowerLite E20</t>
+  </si>
+  <si>
+    <t>Audiovisual</t>
+  </si>
+  <si>
+    <t>Epson</t>
+  </si>
+  <si>
+    <t>EPSE20X7731</t>
+  </si>
+  <si>
+    <t>Auditório</t>
+  </si>
+  <si>
+    <t>Márcia Andrade</t>
+  </si>
+  <si>
+    <t>12/08/2024</t>
+  </si>
+  <si>
+    <t>3.450,00</t>
+  </si>
+  <si>
+    <t>0200005</t>
+  </si>
+  <si>
+    <t>Mesa de reunião oval 2,40 m</t>
+  </si>
+  <si>
+    <t>Sala de Reuniões</t>
+  </si>
+  <si>
     <t>Roberto Farias</t>
-  </si>
-  <si>
-    <t>Novo</t>
-  </si>
-  <si>
-    <t>15/10/2026</t>
-  </si>
-  <si>
-    <t>6.290,00</t>
-  </si>
-  <si>
-    <t>0200002</t>
-  </si>
-  <si>
-    <t>DLT5440A02</t>
-  </si>
-  <si>
-    <t>0200003</t>
-  </si>
-  <si>
-    <t>Cadeira giratória ergonômica com braços</t>
-  </si>
-  <si>
-    <t>Mobiliário</t>
-  </si>
-  <si>
-    <t>Cavaletti</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Secretaria de Administração</t>
-  </si>
-  <si>
-    <t>Márcia Andrade</t>
-  </si>
-  <si>
-    <t>Bom</t>
-  </si>
-  <si>
-    <t>03/03/2025</t>
-  </si>
-  <si>
-    <t>890,00</t>
-  </si>
-  <si>
-    <t>0200004</t>
-  </si>
-  <si>
-    <t>Projetor multimídia Epson PowerLite E20</t>
-  </si>
-  <si>
-    <t>Audiovisual</t>
-  </si>
-  <si>
-    <t>Epson</t>
-  </si>
-  <si>
-    <t>EPSE20X7731</t>
-  </si>
-  <si>
-    <t>Auditório</t>
-  </si>
-  <si>
-    <t>12/08/2024</t>
-  </si>
-  <si>
-    <t>3.450,00</t>
-  </si>
-  <si>
-    <t>0200005</t>
-  </si>
-  <si>
-    <t>Mesa de reunião oval 2,40 m</t>
-  </si>
-  <si>
-    <t>Sala de Reuniões</t>
   </si>
   <si>
     <t>Regular</t>
@@ -642,7 +648,7 @@
         <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
         <v>19</v>
@@ -656,28 +662,28 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
         <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="I4" t="s">
         <v>31</v>
@@ -712,51 +718,51 @@
         <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I5" t="s">
         <v>31</v>
       </c>
       <c r="J5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
         <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Comarca → setor → sala, filtros e solicitações de bens
- Estrutura do Tribunal: unidade = comarca (sede/comarca), setor com tipo
  (vara, gabinete, secretaria…) e sala opcional no bem; importação e
  exportação com as colunas Comarca · Setor · Sala.
- Inventário por setor: varas da mesma comarca em paralelo, sem sobreposição.
- Cobertura por setor no painel (inclui setores ainda sem bens).
- Filtros em bens (marca, responsável, sala, última conferência),
  movimentações (tipo, comarca/setor, pessoa, período) e pendências
  (origem, setor).
- Solicitações de bens: pedir, sugerir bem parado, atender com
  movimentação (fecha sozinho), encaminhar para compra com ofício em PDF,
  recusar e cancelar.
- Seed: Comarca de Marabá + persona do interior (Juliana); completa o que
  falta num banco já no ar sem apagar nada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/novos_itens_predio_sede.xlsx
+++ b/sample-data/novos_itens_predio_sede.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
   <si>
     <t>Nº Tombamento</t>
   </si>
@@ -28,10 +28,13 @@
     <t>Nº de Série</t>
   </si>
   <si>
-    <t>Unidade</t>
-  </si>
-  <si>
-    <t>Localização</t>
+    <t>Comarca</t>
+  </si>
+  <si>
+    <t>Setor</t>
+  </si>
+  <si>
+    <t>Sala</t>
   </si>
   <si>
     <t>Responsável</t>
@@ -67,6 +70,9 @@
     <t>Secretaria de Informática</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Paula Menezes</t>
   </si>
   <si>
@@ -98,9 +104,6 @@
   </si>
   <si>
     <t>Cavaletti</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Secretaria de Administração</t>
@@ -541,21 +544,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="5" width="14" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
+    <col min="8" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,104 +594,113 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
         <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>32</v>
@@ -694,63 +708,69 @@
       <c r="K4" t="s">
         <v>33</v>
       </c>
+      <c r="L4" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
         <v>40</v>
       </c>
       <c r="I5" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="K5" t="s">
         <v>42</v>
       </c>
+      <c r="L5" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="H6" t="s">
         <v>46</v>
@@ -763,6 +783,9 @@
       </c>
       <c r="K6" t="s">
         <v>49</v>
+      </c>
+      <c r="L6" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>